<commit_message>
Merge latest changes from origin/tejas
</commit_message>
<xml_diff>
--- a/backend/app/data/updated_scheduling_data.xlsx
+++ b/backend/app/data/updated_scheduling_data.xlsx
@@ -913,7 +913,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -3335,7 +3335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="3">
@@ -3595,6 +3595,58 @@
       <c r="J5" s="2" t="inlineStr">
         <is>
           <t>https://meet.onboardiq.io/session/pNt8Yi7y</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Prathamesh</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>HR Introduction</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Shivani</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>11 Apr</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>11:00 AM</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>confirmed</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-09 07:40:40 UTC</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>https://meet.onboardiq.io/session/dkro0X7A</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Email reply issue resolved successfully
</commit_message>
<xml_diff>
--- a/backend/app/data/updated_scheduling_data.xlsx
+++ b/backend/app/data/updated_scheduling_data.xlsx
@@ -657,7 +657,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -3335,7 +3335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="3">
@@ -3959,6 +3959,58 @@
       <c r="J12" s="2" t="inlineStr">
         <is>
           <t>https://meet.onboardiq.io/session/lM33oMSQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Tejas Ninawe</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>HR Introduction</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Mohini</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>10 Apr</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>04:30 PM</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>confirmed</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-15 05:21:08 UTC</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>https://meet.onboardiq.io/session/GCWPSoNW</t>
         </is>
       </c>
     </row>

</xml_diff>